<commit_message>
add sertifikat kelulusan testcase
</commit_message>
<xml_diff>
--- a/inputan.xlsx
+++ b/inputan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Personal\Katalon Studio\Sisfo Bahasa Remake\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/agungtrisnaa/Katalon Studio/Sisfo-Bahasa-Remake/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3079DBA1-6B1C-48F2-8159-083031BC25F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FD82207-7421-A14D-B69A-3FBF43905F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24525" yWindow="3735" windowWidth="21600" windowHeight="11295" xr2:uid="{B515BAB2-BCAD-4B7E-AD5C-E3DAB4375D2E}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19660" xr2:uid="{B515BAB2-BCAD-4B7E-AD5C-E3DAB4375D2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Link</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t>IDsiswa</t>
+  </si>
+  <si>
+    <t>nSertif</t>
   </si>
 </sst>
 </file>
@@ -516,31 +519,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5B4298E-1260-483C-BDCD-A0BAF6E7D4E6}">
-  <dimension ref="A1:V8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:W8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.28515625" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.33203125" customWidth="1"/>
+    <col min="5" max="5" width="19.5" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" customWidth="1"/>
-    <col min="12" max="12" width="14.42578125" customWidth="1"/>
-    <col min="13" max="13" width="12.28515625" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" customWidth="1"/>
-    <col min="16" max="16" width="14.5703125" customWidth="1"/>
-    <col min="17" max="17" width="19.7109375" customWidth="1"/>
-    <col min="18" max="18" width="15.28515625" customWidth="1"/>
-    <col min="19" max="19" width="25.42578125" customWidth="1"/>
-    <col min="22" max="22" width="11.28515625" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" customWidth="1"/>
+    <col min="12" max="12" width="14.5" customWidth="1"/>
+    <col min="13" max="13" width="12.33203125" customWidth="1"/>
+    <col min="14" max="14" width="12.1640625" customWidth="1"/>
+    <col min="16" max="16" width="14.5" customWidth="1"/>
+    <col min="17" max="17" width="19.6640625" customWidth="1"/>
+    <col min="18" max="18" width="15.33203125" customWidth="1"/>
+    <col min="19" max="19" width="25.5" customWidth="1"/>
+    <col min="22" max="22" width="11.33203125" customWidth="1"/>
+    <col min="23" max="23" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -607,8 +611,11 @@
       <c r="V1" t="s">
         <v>37</v>
       </c>
+      <c r="W1" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -675,8 +682,11 @@
       <c r="V2">
         <v>1205497852</v>
       </c>
+      <c r="W2">
+        <v>17343643723</v>
+      </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="D8" s="3"/>
     </row>
   </sheetData>

</xml_diff>